<commit_message>
RNA-seq: full FTP manifest (324 files, 6.5 TiB); S3->FTP fallback for mirror gaps
S3 mirror lacks 6.3 TiB of RNA-seq (Illumina/Iso-Seq/Baylor) and 2.1 TiB of
Element AVITI 2024-09, verified against FTP current.tree.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAB_HG_Catalog.xlsx
+++ b/GIAB_HG_Catalog.xlsx
@@ -134,7 +134,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -191,8 +191,13 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -214,11 +219,12 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -299,6 +305,31 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1065,7 +1096,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>data/ChineseTrio/HG006_NA24694_father/</t>
+          <t>data/ChineseTrio/HG006_NA24694-huCA017E_father/</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1133,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>data/ChineseTrio/HG007_NA24695_mother/</t>
+          <t>data/ChineseTrio/HG007_NA24695-hu38168_mother/</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1322,7 +1353,7 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1384,7 +1415,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1419,14 +1450,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H6" s="21" t="inlineStr"/>
-      <c r="I6" s="21" t="inlineStr"/>
-      <c r="J6" s="21" t="inlineStr"/>
-      <c r="K6" s="21" t="inlineStr"/>
-      <c r="L6" s="21" t="inlineStr"/>
+      <c r="H6" s="35" t="n"/>
+      <c r="I6" s="35" t="n"/>
+      <c r="J6" s="35" t="n"/>
+      <c r="K6" s="35" t="n"/>
+      <c r="L6" s="35" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1471,842 +1502,1257 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J7" s="21" t="inlineStr"/>
-      <c r="K7" s="21" t="inlineStr"/>
-      <c r="L7" s="21" t="inlineStr"/>
+      <c r="J7" s="35" t="n"/>
+      <c r="K7" s="35" t="n"/>
+      <c r="L7" s="35" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>Short-read</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>BGISEQ-500 / MGISEQ (DNBSEQ, BGI/MGI)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J8" s="35" t="n"/>
+      <c r="K8" s="35" t="n"/>
+      <c r="L8" s="35" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Illumina synthetic long reads (Moleculo / read clouds)</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr"/>
-      <c r="K8" s="21" t="inlineStr"/>
-      <c r="L8" s="21" t="inlineStr"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J9" s="35" t="n"/>
+      <c r="K9" s="35" t="n"/>
+      <c r="L9" s="35" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>10x Genomics linked-reads (GemCode/Chromium)</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H9" s="22" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I9" s="22" t="inlineStr">
+      <c r="I10" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J9" s="21" t="inlineStr"/>
-      <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="21" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="J10" s="35" t="n"/>
+      <c r="K10" s="35" t="n"/>
+      <c r="L10" s="35" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>Linked/synthetic</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>stLFR (single-tube long fragment read, BGI/MGI)</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="35" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Complete Genomics WGS (standard)</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J10" s="21" t="inlineStr"/>
-      <c r="K10" s="21" t="inlineStr"/>
-      <c r="L10" s="21" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="n"/>
+      <c r="K12" s="35" t="n"/>
+      <c r="L12" s="35" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Complete Genomics LFR</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F11" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G11" s="21" t="inlineStr"/>
-      <c r="H11" s="21" t="inlineStr"/>
-      <c r="I11" s="21" t="inlineStr"/>
-      <c r="J11" s="21" t="inlineStr"/>
-      <c r="K11" s="21" t="inlineStr"/>
-      <c r="L11" s="21" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G13" s="35" t="n"/>
+      <c r="H13" s="35" t="n"/>
+      <c r="I13" s="35" t="n"/>
+      <c r="J13" s="35" t="n"/>
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="35" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Ion Torrent / Ion Proton exome</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="inlineStr"/>
-      <c r="I12" s="21" t="inlineStr"/>
-      <c r="J12" s="21" t="inlineStr"/>
-      <c r="K12" s="21" t="inlineStr"/>
-      <c r="L12" s="21" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H14" s="35" t="n"/>
+      <c r="I14" s="35" t="n"/>
+      <c r="J14" s="35" t="n"/>
+      <c r="K14" s="35" t="n"/>
+      <c r="L14" s="35" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>SOLiD WGS</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr"/>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr"/>
-      <c r="F13" s="21" t="inlineStr"/>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H13" s="21" t="inlineStr"/>
-      <c r="I13" s="21" t="inlineStr"/>
-      <c r="J13" s="21" t="inlineStr"/>
-      <c r="K13" s="21" t="inlineStr"/>
-      <c r="L13" s="21" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H15" s="35" t="n"/>
+      <c r="I15" s="35" t="n"/>
+      <c r="J15" s="35" t="n"/>
+      <c r="K15" s="35" t="n"/>
+      <c r="L15" s="35" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="37" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>PacBio CLR (RS II / Sequel)</t>
         </is>
       </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I14" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J14" s="21" t="inlineStr"/>
-      <c r="K14" s="21" t="inlineStr"/>
-      <c r="L14" s="21" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J16" s="35" t="n"/>
+      <c r="K16" s="35" t="n"/>
+      <c r="L16" s="35" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>PacBio HiFi / CCS (Sequel II / Revio)</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr">
+      <c r="I17" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Oxford Nanopore (PromethION/MinION, incl. ultra-long)</t>
         </is>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="I18" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Bionano optical mapping (Saphyr/Irys)</t>
         </is>
       </c>
-      <c r="C17" s="22" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H17" s="22" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I17" s="22" t="inlineStr">
+      <c r="I19" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K17" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L17" s="22" t="inlineStr">
+      <c r="J19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L19" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="25" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="38" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Strand-seq</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr"/>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr"/>
-      <c r="F18" s="21" t="inlineStr"/>
-      <c r="G18" s="21" t="inlineStr"/>
-      <c r="H18" s="21" t="inlineStr"/>
-      <c r="I18" s="21" t="inlineStr"/>
-      <c r="J18" s="21" t="inlineStr"/>
-      <c r="K18" s="21" t="inlineStr"/>
-      <c r="L18" s="21" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I20" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J20" s="35" t="n"/>
+      <c r="K20" s="35" t="n"/>
+      <c r="L20" s="35" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Hi-C (Arima / Phase / Dovetail)</t>
-        </is>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Hi-C (Arima / Phase / Dovetail / UCSC)</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E19" s="21" t="inlineStr"/>
-      <c r="F19" s="21" t="inlineStr"/>
-      <c r="G19" s="21" t="inlineStr"/>
-      <c r="H19" s="21" t="inlineStr"/>
-      <c r="I19" s="21" t="inlineStr"/>
-      <c r="J19" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K19" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L19" s="21" t="inlineStr"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G21" s="35" t="n"/>
+      <c r="H21" s="35" t="n"/>
+      <c r="I21" s="35" t="n"/>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L21" s="35" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Element Biosciences AVITI</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr"/>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr"/>
-      <c r="F20" s="21" t="inlineStr"/>
-      <c r="G20" s="21" t="inlineStr"/>
-      <c r="H20" s="21" t="inlineStr"/>
-      <c r="I20" s="21" t="inlineStr"/>
-      <c r="J20" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K20" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L20" s="22" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H22" s="35" t="n"/>
+      <c r="I22" s="35" t="n"/>
+      <c r="J22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L22" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Ultima Genomics UG100</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr"/>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr"/>
-      <c r="F21" s="21" t="inlineStr"/>
-      <c r="G21" s="21" t="inlineStr"/>
-      <c r="H21" s="21" t="inlineStr"/>
-      <c r="I21" s="21" t="inlineStr"/>
-      <c r="J21" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K21" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L21" s="21" t="inlineStr"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E23" s="35" t="n"/>
+      <c r="F23" s="35" t="n"/>
+      <c r="G23" s="35" t="n"/>
+      <c r="H23" s="35" t="n"/>
+      <c r="I23" s="35" t="n"/>
+      <c r="J23" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L23" s="35" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>PacBio Onso (SBB short-read)</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr"/>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr"/>
-      <c r="F22" s="21" t="inlineStr"/>
-      <c r="G22" s="21" t="inlineStr"/>
-      <c r="H22" s="21" t="inlineStr"/>
-      <c r="I22" s="21" t="inlineStr"/>
-      <c r="J22" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K22" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L22" s="22" t="inlineStr">
+      <c r="E24" s="35" t="n"/>
+      <c r="F24" s="35" t="n"/>
+      <c r="G24" s="35" t="n"/>
+      <c r="H24" s="35" t="n"/>
+      <c r="I24" s="35" t="n"/>
+      <c r="J24" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L24" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="38" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>Cytogenetics: karyotype / KromaTiD dGH</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr"/>
-      <c r="D23" s="21" t="inlineStr"/>
-      <c r="E23" s="21" t="inlineStr"/>
-      <c r="F23" s="21" t="inlineStr"/>
-      <c r="G23" s="21" t="inlineStr"/>
-      <c r="H23" s="21" t="inlineStr"/>
-      <c r="I23" s="21" t="inlineStr"/>
-      <c r="J23" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K23" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L23" s="21" t="inlineStr"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="35" t="n"/>
+      <c r="G25" s="35" t="n"/>
+      <c r="H25" s="35" t="n"/>
+      <c r="I25" s="35" t="n"/>
+      <c r="J25" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L25" s="35" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Single-cell WGS (BioSkryb)</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr"/>
-      <c r="D24" s="21" t="inlineStr"/>
-      <c r="E24" s="21" t="inlineStr"/>
-      <c r="F24" s="21" t="inlineStr"/>
-      <c r="G24" s="21" t="inlineStr"/>
-      <c r="H24" s="21" t="inlineStr"/>
-      <c r="I24" s="21" t="inlineStr"/>
-      <c r="J24" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K24" s="20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L24" s="21" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Single-cell WGS (BioSkryb ResolveDNA)</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+      <c r="F26" s="35" t="n"/>
+      <c r="G26" s="35" t="n"/>
+      <c r="H26" s="35" t="n"/>
+      <c r="I26" s="35" t="n"/>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L26" s="35" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Illumina bulk RNA-seq (mRNA + total RNA, UNC ×3 replicate)</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H27" s="35" t="n"/>
+      <c r="I27" s="35" t="n"/>
+      <c r="J27" s="35" t="n"/>
+      <c r="K27" s="35" t="n"/>
+      <c r="L27" s="35" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Illumina mRNA + lncRNA (Google/Novogene)</t>
+        </is>
+      </c>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G28" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H28" s="35" t="n"/>
+      <c r="I28" s="35" t="n"/>
+      <c r="J28" s="35" t="n"/>
+      <c r="K28" s="35" t="n"/>
+      <c r="L28" s="35" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>PacBio Iso-Seq (Sequel II subreads, Google)</t>
+        </is>
+      </c>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E29" s="35" t="n"/>
+      <c r="F29" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H29" s="35" t="n"/>
+      <c r="I29" s="35" t="n"/>
+      <c r="J29" s="35" t="n"/>
+      <c r="K29" s="35" t="n"/>
+      <c r="L29" s="35" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>PacBio MAS-Seq / Kinnex (full-length isoform)</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G30" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H30" s="35" t="n"/>
+      <c r="I30" s="35" t="n"/>
+      <c r="J30" s="35" t="n"/>
+      <c r="K30" s="35" t="n"/>
+      <c r="L30" s="35" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>PacBio HiFi RNA (Baylor)</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E31" s="35" t="n"/>
+      <c r="F31" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G31" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H31" s="35" t="n"/>
+      <c r="I31" s="35" t="n"/>
+      <c r="J31" s="35" t="n"/>
+      <c r="K31" s="35" t="n"/>
+      <c r="L31" s="35" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>RNA-seq</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>ONT direct RNA (Mason)</t>
+        </is>
+      </c>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E32" s="35" t="n"/>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G32" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H32" s="35" t="n"/>
+      <c r="I32" s="35" t="n"/>
+      <c r="J32" s="35" t="n"/>
+      <c r="K32" s="35" t="n"/>
+      <c r="L32" s="35" t="n"/>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="40" t="n"/>
+      <c r="B33" s="40" t="n"/>
+      <c r="C33" s="40" t="n"/>
+      <c r="D33" s="40" t="n"/>
+      <c r="E33" s="40" t="n"/>
+      <c r="F33" s="40" t="n"/>
+      <c r="G33" s="40" t="n"/>
+      <c r="H33" s="40" t="n"/>
+      <c r="I33" s="40" t="n"/>
+      <c r="J33" s="40" t="n"/>
+      <c r="K33" s="40" t="n"/>
+      <c r="L33" s="40" t="n"/>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="40" t="n"/>
+      <c r="B34" s="41" t="inlineStr">
         <is>
           <t>플랫폼 수 (Y+L)</t>
         </is>
       </c>
-      <c r="C26" s="27" t="n">
-        <v>13</v>
-      </c>
-      <c r="D26" s="27" t="n">
-        <v>18</v>
-      </c>
-      <c r="E26" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="G26" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="H26" s="27" t="n">
-        <v>9</v>
-      </c>
-      <c r="I26" s="27" t="n">
-        <v>9</v>
-      </c>
-      <c r="J26" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="K26" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="L26" s="27" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="C34" s="8">
+        <f>COUNTA(C5:C32)</f>
+        <v/>
+      </c>
+      <c r="D34" s="8">
+        <f>COUNTA(D5:D32)</f>
+        <v/>
+      </c>
+      <c r="E34" s="8">
+        <f>COUNTA(E5:E32)</f>
+        <v/>
+      </c>
+      <c r="F34" s="8">
+        <f>COUNTA(F5:F32)</f>
+        <v/>
+      </c>
+      <c r="G34" s="8">
+        <f>COUNTA(G5:G32)</f>
+        <v/>
+      </c>
+      <c r="H34" s="8">
+        <f>COUNTA(H5:H32)</f>
+        <v/>
+      </c>
+      <c r="I34" s="8">
+        <f>COUNTA(I5:I32)</f>
+        <v/>
+      </c>
+      <c r="J34" s="8">
+        <f>COUNTA(J5:J32)</f>
+        <v/>
+      </c>
+      <c r="K34" s="8">
+        <f>COUNTA(K5:K32)</f>
+        <v/>
+      </c>
+      <c r="L34" s="8">
+        <f>COUNTA(L5:L32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="40" t="n"/>
+      <c r="B35" s="40" t="n"/>
+      <c r="C35" s="40" t="n"/>
+      <c r="D35" s="40" t="n"/>
+      <c r="E35" s="40" t="n"/>
+      <c r="F35" s="40" t="n"/>
+      <c r="G35" s="40" t="n"/>
+      <c r="H35" s="40" t="n"/>
+      <c r="I35" s="40" t="n"/>
+      <c r="J35" s="40" t="n"/>
+      <c r="K35" s="40" t="n"/>
+      <c r="L35" s="40" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>· 범례: Y = 데이터 제공, L = 제한적/일부 제공, 빈칸 = 알려진 데이터 없음.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="29" t="inlineStr">
-        <is>
-          <t>· 본 매트릭스는 GIAB 공개 논문·NIST 문서 및 공식 data index를 근거로 '플랫폼 단위' 가용성을 요약한 것으로, 실제 파일 존재 여부·커버리지·최신 추가분은 아래 GIAB FTP 및 data index에서 최종 확인해야 한다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
-        <is>
-          <t>· HG002는 사실상 모든 신규 플랫폼이 우선 적용되는 대표 샘플이라 커버리지가 가장 넓고, trio 부모(HG003/4, HG006/7)는 일부 신규 플랫폼이 제한적이다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="29" t="inlineStr">
-        <is>
-          <t>· HG008(종양-정상)은 2024~2025년 최신 기술 중심의 체세포 벤치마크로, 구형 플랫폼(SOLiD/CG/Ion 등)은 포함하지 않는다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="29" t="inlineStr">
-        <is>
-          <t>· HG008 정상은 십이지장(HG008-N-D)과 췌장(HG008-N-P) 두 조직으로, N-D가 주(primary) 정상 대조군으로 더 많은 플랫폼에서 깊이 시퀀싱되었고 N-P는 핵심 WGS 위주의 보조 샘플이다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="29" t="inlineStr">
-        <is>
-          <t>· 표준 GIAB 벤치마크 샘플은 HG001–HG008이며(HG008은 T·N-D·N-P의 3개 물리 샘플), HG009 이상 신규 샘플은 확보·컨센트 확대가 진행 중이나 아직 정식 번호·릴리스가 부여되지 않았다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="29" t="inlineStr">
-        <is>
-          <t>· 생식세포(HG001–HG007) 데이터는 계속 갱신되므로, Illumina/PacBio HiFi/ONT 등은 표기보다 더 많은 데이터가 있을 수 있다.</t>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>· 범례: Y = 데이터 제공, L = 제한적/일부, 빈칸 = 알려진 데이터 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>· 이 시트는 2026-08-13 기준 GIAB FTP 전체 파일목록(current.tree, 86,392개)과 S3 버킷 실시간 목록(87,527개)을 대조해 검증했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>· 2026-08-13 보정: SOLiD(HG001), Strand-seq(HG003~HG007), Hi-C(HG003·HG004), Element AVITI(HG001·HG003~HG005)를 빈칸에서 Y로 수정. BGISEQ/MGISEQ와 stLFR 행을 신규 추가(7개 germline 전체 제공).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>· RNA-seq는 HG002·HG004·HG005 3개 샘플만 존재하며 총 6.5 TiB(324 files)다. HG001·HG003·HG006·HG007과 HG008(종양-정상)에는 RNA 데이터가 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>· 주의: RNA-seq 중 Illumina(UNC·Google)·Iso-Seq·Baylor HiFi RNA는 FTP에만 있고 AWS S3 미러에는 없다(6.3 TiB 누락). 이 데이터는 wget/FTP로 받아야 한다. MAS-Seq와 ONT direct RNA만 S3에 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>· 주의: germline DNA에서도 Element AVITI 2024-09(HG001~HG005, 약 2.1 TiB)는 S3 미러 누락 상태이며 FTP에서만 받을 수 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>· GIAB 공식 배포에 single-cell RNA-seq과 small RNA-seq(miRNA)은 없다. Single-cell은 DNA 기반(Strand-seq, BioSkryb)뿐이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>· HG002는 사실상 모든 신규 플랫폼이 우선 적용되는 대표 샘플이고, trio 부모(HG003/4, HG006/7)는 일부 신규 플랫폼이 미적용이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>· HG008(종양-정상)은 2024~2025년 최신 기기 중심의 체세포 벤치마크로, 구형 플랫폼(SOLiD/CG/Ion 등)은 제공되지 않는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>· 표준 GIAB 벤치마크 샘플은 HG001~HG008이며(HG008은 T·N-D·N-P의 3개 하위 시료), HG009 이상 신규 샘플은 확정·공표되지 않았다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A30:L30"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A33:L33"/>
-    <mergeCell ref="A32:L32"/>
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="A34:L34"/>
-    <mergeCell ref="A35:L35"/>
+  <mergeCells count="10">
+    <mergeCell ref="A38:L38"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="A46:L46"/>
+    <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A39:L39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2318,7 +2764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2552,6 +2998,56 @@
       <c r="B23" s="33" t="inlineStr">
         <is>
           <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/data_somatic/HG008/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>추가 경로 (2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="42" t="inlineStr">
+        <is>
+          <t>RNA-seq 데이터 FTP (HG002/HG004/HG005)</t>
+        </is>
+      </c>
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/data_RNAseq/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>AWS S3 미러 (일부 데이터 누락 — 아래 주의)</t>
+        </is>
+      </c>
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t>https://giab.s3.amazonaws.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>FTP 전체 파일목록 (크기·MD5 포함)</t>
+        </is>
+      </c>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/current.tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>· S3 미러는 FTP보다 불완전하다. RNA-seq Illumina/Iso-Seq(6.3 TiB)과 Element AVITI 2024-09(2.1 TiB)은 S3에 없으므로 FTP(wget)로 받아야 한다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add HG009 + all S3-missing data to manifests (HEAD-verified); harden resume
- manifests/HG009/pacbio_hifi.tsv: new tumor-normal benchmark (563 files, 1.5 TiB)
- Merge 4,504 HEAD-verified FTP-only files into per-sample manifests
  (HG008 other_passages/ILMN-WGS/Dovetail, Element AVITI 2024-09,
   HG002B PhaseGenomics Hi-C, HG001 haplotagged BAMs, release old versions)
- New trio_analysis category (HG002 T2T-Q100 draft benchmarks, 59 GiB)
- verify.sh: add HG009 to ALL_SAMPLES (blocker: HG009 progress was invisible),
  guard empty manifest match
- download.sh: FTP fallback also on S3 size mismatch; clean orphan .part
- run_priority.sh: include trio_analysis + rnaseq in default order
- README: totals now 115.6 TB / 76,595 files, ETA at measured 83 MB/s

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAB_HG_Catalog.xlsx
+++ b/GIAB_HG_Catalog.xlsx
@@ -134,7 +134,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -193,6 +193,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="002F5F41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
@@ -224,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -305,6 +310,9 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -320,7 +328,7 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -695,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -722,6 +730,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr"/>
     </row>
@@ -790,7 +799,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>· 'Platform Matrix' : 샘플 × 시퀀싱 플랫폼 가용성 매트릭스 (Y/L/빈칸)</t>
+          <t>· 'Platform Matrix' : 샘플 × 시퀀싱 플랫폼 가용성 매트릭스 (Y/L/빈칸). DNA 22종 + RNA-seq 6종, HG001~HG009</t>
         </is>
       </c>
     </row>
@@ -822,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1248,6 +1257,80 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>HG009-T</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>HTB3066 유래 종양 세포주 (계대·클론)</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>HG009 Tumor-Normal</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>종양 (tumor)</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>세포주 기반 종양</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>GIAB 두 번째 체세포 벤치마크(2026-07 공개). bulk 계대 p16·p42와 클론 6종(1C3·1D5·3C4·3C9·3F2·4G9)을 제공하며, 계대·클론 간 비교로 체세포 변이 검출을 평가하도록 설계됐다. 현재 PacBio HiFi Revio(SPRQ)만 제공.</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>data_somatic/HG009/NIST/HG009-T_bulk/, .../HG009-T_clones/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>HG009-N</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>동일 개체 정상 세포주 (WT·LVTert)</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>HG009 Tumor-Normal</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>정상 (normal)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>세포주 기반 정상</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>HG009-T와 짝을 이루는 정상 시료. WT 계대 p4·p25와 hTERT 불멸화 라인(LVTert-p23)을 제공한다. 정상-정상 비교(p25 vs p4)로 위양성 평가가 가능하다.</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>data_somatic/HG009/NIST/HG009-N_bulk/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1259,21 +1342,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9.5" customWidth="1" min="3" max="3"/>
+    <col width="9.5" customWidth="1" min="4" max="4"/>
+    <col width="9.5" customWidth="1" min="5" max="5"/>
+    <col width="9.5" customWidth="1" min="6" max="6"/>
+    <col width="9.5" customWidth="1" min="7" max="7"/>
+    <col width="9.5" customWidth="1" min="8" max="8"/>
+    <col width="9.5" customWidth="1" min="9" max="9"/>
+    <col width="9.5" customWidth="1" min="10" max="10"/>
+    <col width="9.5" customWidth="1" min="11" max="11"/>
+    <col width="9.5" customWidth="1" min="12" max="12"/>
+    <col width="9.5" customWidth="1" min="13" max="13"/>
+    <col width="9.5" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1351,9 +1436,19 @@
           <t>HG008-N-P</t>
         </is>
       </c>
+      <c r="M4" s="34" t="inlineStr">
+        <is>
+          <t>HG009-T</t>
+        </is>
+      </c>
+      <c r="N4" s="34" t="inlineStr">
+        <is>
+          <t>HG009-N</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1413,9 +1508,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="M5" s="36" t="n"/>
+      <c r="N5" s="36" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1450,14 +1547,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H6" s="35" t="n"/>
-      <c r="I6" s="35" t="n"/>
-      <c r="J6" s="35" t="n"/>
-      <c r="K6" s="35" t="n"/>
-      <c r="L6" s="35" t="n"/>
+      <c r="H6" s="36" t="n"/>
+      <c r="I6" s="36" t="n"/>
+      <c r="J6" s="36" t="n"/>
+      <c r="K6" s="36" t="n"/>
+      <c r="L6" s="36" t="n"/>
+      <c r="M6" s="36" t="n"/>
+      <c r="N6" s="36" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1502,12 +1601,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J7" s="35" t="n"/>
-      <c r="K7" s="35" t="n"/>
-      <c r="L7" s="35" t="n"/>
+      <c r="J7" s="36" t="n"/>
+      <c r="K7" s="36" t="n"/>
+      <c r="L7" s="36" t="n"/>
+      <c r="M7" s="36" t="n"/>
+      <c r="N7" s="36" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1552,12 +1653,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J8" s="35" t="n"/>
-      <c r="K8" s="35" t="n"/>
-      <c r="L8" s="35" t="n"/>
+      <c r="J8" s="36" t="n"/>
+      <c r="K8" s="36" t="n"/>
+      <c r="L8" s="36" t="n"/>
+      <c r="M8" s="36" t="n"/>
+      <c r="N8" s="36" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
@@ -1602,12 +1705,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J9" s="35" t="n"/>
-      <c r="K9" s="35" t="n"/>
-      <c r="L9" s="35" t="n"/>
+      <c r="J9" s="36" t="n"/>
+      <c r="K9" s="36" t="n"/>
+      <c r="L9" s="36" t="n"/>
+      <c r="M9" s="36" t="n"/>
+      <c r="N9" s="36" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
@@ -1652,12 +1757,14 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J10" s="35" t="n"/>
-      <c r="K10" s="35" t="n"/>
-      <c r="L10" s="35" t="n"/>
+      <c r="J10" s="36" t="n"/>
+      <c r="K10" s="36" t="n"/>
+      <c r="L10" s="36" t="n"/>
+      <c r="M10" s="36" t="n"/>
+      <c r="N10" s="36" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="36" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
@@ -1702,12 +1809,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J11" s="35" t="n"/>
-      <c r="K11" s="35" t="n"/>
-      <c r="L11" s="35" t="n"/>
+      <c r="J11" s="36" t="n"/>
+      <c r="K11" s="36" t="n"/>
+      <c r="L11" s="36" t="n"/>
+      <c r="M11" s="36" t="n"/>
+      <c r="N11" s="36" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="34" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1752,12 +1861,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J12" s="35" t="n"/>
-      <c r="K12" s="35" t="n"/>
-      <c r="L12" s="35" t="n"/>
+      <c r="J12" s="36" t="n"/>
+      <c r="K12" s="36" t="n"/>
+      <c r="L12" s="36" t="n"/>
+      <c r="M12" s="36" t="n"/>
+      <c r="N12" s="36" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="36" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>Linked/synthetic</t>
         </is>
@@ -1787,15 +1898,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="35" t="n"/>
-      <c r="I13" s="35" t="n"/>
-      <c r="J13" s="35" t="n"/>
-      <c r="K13" s="35" t="n"/>
-      <c r="L13" s="35" t="n"/>
+      <c r="G13" s="36" t="n"/>
+      <c r="H13" s="36" t="n"/>
+      <c r="I13" s="36" t="n"/>
+      <c r="J13" s="36" t="n"/>
+      <c r="K13" s="36" t="n"/>
+      <c r="L13" s="36" t="n"/>
+      <c r="M13" s="36" t="n"/>
+      <c r="N13" s="36" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1830,14 +1943,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="35" t="n"/>
-      <c r="J14" s="35" t="n"/>
-      <c r="K14" s="35" t="n"/>
-      <c r="L14" s="35" t="n"/>
+      <c r="H14" s="36" t="n"/>
+      <c r="I14" s="36" t="n"/>
+      <c r="J14" s="36" t="n"/>
+      <c r="K14" s="36" t="n"/>
+      <c r="L14" s="36" t="n"/>
+      <c r="M14" s="36" t="n"/>
+      <c r="N14" s="36" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="34" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -1857,21 +1972,23 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="35" t="n"/>
+      <c r="E15" s="36" t="n"/>
+      <c r="F15" s="36" t="n"/>
       <c r="G15" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" s="35" t="n"/>
-      <c r="I15" s="35" t="n"/>
-      <c r="J15" s="35" t="n"/>
-      <c r="K15" s="35" t="n"/>
-      <c r="L15" s="35" t="n"/>
+      <c r="H15" s="36" t="n"/>
+      <c r="I15" s="36" t="n"/>
+      <c r="J15" s="36" t="n"/>
+      <c r="K15" s="36" t="n"/>
+      <c r="L15" s="36" t="n"/>
+      <c r="M15" s="36" t="n"/>
+      <c r="N15" s="36" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="37" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
@@ -1916,12 +2033,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J16" s="35" t="n"/>
-      <c r="K16" s="35" t="n"/>
-      <c r="L16" s="35" t="n"/>
+      <c r="J16" s="36" t="n"/>
+      <c r="K16" s="36" t="n"/>
+      <c r="L16" s="36" t="n"/>
+      <c r="M16" s="36" t="n"/>
+      <c r="N16" s="36" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
@@ -1981,9 +2100,19 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="M17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="37" t="inlineStr">
+      <c r="A18" s="38" t="inlineStr">
         <is>
           <t>Long-read</t>
         </is>
@@ -2043,9 +2172,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="M18" s="36" t="n"/>
+      <c r="N18" s="36" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="38" t="inlineStr">
+      <c r="A19" s="39" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
@@ -2105,9 +2236,11 @@
           <t>L</t>
         </is>
       </c>
+      <c r="M19" s="36" t="n"/>
+      <c r="N19" s="36" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="38" t="inlineStr">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
@@ -2117,7 +2250,7 @@
           <t>Strand-seq</t>
         </is>
       </c>
-      <c r="C20" s="35" t="n"/>
+      <c r="C20" s="36" t="n"/>
       <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2148,19 +2281,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J20" s="35" t="n"/>
-      <c r="K20" s="35" t="n"/>
-      <c r="L20" s="35" t="n"/>
+      <c r="J20" s="36" t="n"/>
+      <c r="K20" s="36" t="n"/>
+      <c r="L20" s="36" t="n"/>
+      <c r="M20" s="36" t="n"/>
+      <c r="N20" s="36" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="38" t="inlineStr">
+      <c r="A21" s="39" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>Hi-C (Arima / Phase / Dovetail / UCSC)</t>
+          <t>Hi-C / proximity ligation (Arima·Phase·Dovetail·UCSC)</t>
         </is>
       </c>
       <c r="C21" s="22" t="inlineStr">
@@ -2183,9 +2318,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G21" s="35" t="n"/>
-      <c r="H21" s="35" t="n"/>
-      <c r="I21" s="35" t="n"/>
+      <c r="G21" s="36" t="n"/>
+      <c r="H21" s="36" t="n"/>
+      <c r="I21" s="36" t="n"/>
       <c r="J21" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2196,10 +2331,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L21" s="35" t="n"/>
+      <c r="L21" s="20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M21" s="36" t="n"/>
+      <c r="N21" s="36" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -2234,8 +2375,8 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H22" s="35" t="n"/>
-      <c r="I22" s="35" t="n"/>
+      <c r="H22" s="36" t="n"/>
+      <c r="I22" s="36" t="n"/>
       <c r="J22" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2251,9 +2392,11 @@
           <t>L</t>
         </is>
       </c>
+      <c r="M22" s="36" t="n"/>
+      <c r="N22" s="36" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -2263,17 +2406,17 @@
           <t>Ultima Genomics UG100</t>
         </is>
       </c>
-      <c r="C23" s="35" t="n"/>
+      <c r="C23" s="36" t="n"/>
       <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E23" s="35" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="35" t="n"/>
-      <c r="H23" s="35" t="n"/>
-      <c r="I23" s="35" t="n"/>
+      <c r="E23" s="36" t="n"/>
+      <c r="F23" s="36" t="n"/>
+      <c r="G23" s="36" t="n"/>
+      <c r="H23" s="36" t="n"/>
+      <c r="I23" s="36" t="n"/>
       <c r="J23" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2284,10 +2427,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L23" s="35" t="n"/>
+      <c r="L23" s="36" t="n"/>
+      <c r="M23" s="36" t="n"/>
+      <c r="N23" s="36" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="34" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -2297,17 +2442,17 @@
           <t>PacBio Onso (SBB short-read)</t>
         </is>
       </c>
-      <c r="C24" s="35" t="n"/>
+      <c r="C24" s="36" t="n"/>
       <c r="D24" s="22" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="35" t="n"/>
-      <c r="H24" s="35" t="n"/>
-      <c r="I24" s="35" t="n"/>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="36" t="n"/>
+      <c r="G24" s="36" t="n"/>
+      <c r="H24" s="36" t="n"/>
+      <c r="I24" s="36" t="n"/>
       <c r="J24" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2323,9 +2468,11 @@
           <t>L</t>
         </is>
       </c>
+      <c r="M24" s="36" t="n"/>
+      <c r="N24" s="36" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="38" t="inlineStr">
+      <c r="A25" s="39" t="inlineStr">
         <is>
           <t>Optical/other</t>
         </is>
@@ -2335,13 +2482,13 @@
           <t>Cytogenetics: karyotype / KromaTiD dGH</t>
         </is>
       </c>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="35" t="n"/>
-      <c r="E25" s="35" t="n"/>
-      <c r="F25" s="35" t="n"/>
-      <c r="G25" s="35" t="n"/>
-      <c r="H25" s="35" t="n"/>
-      <c r="I25" s="35" t="n"/>
+      <c r="C25" s="36" t="n"/>
+      <c r="D25" s="36" t="n"/>
+      <c r="E25" s="36" t="n"/>
+      <c r="F25" s="36" t="n"/>
+      <c r="G25" s="36" t="n"/>
+      <c r="H25" s="36" t="n"/>
+      <c r="I25" s="36" t="n"/>
       <c r="J25" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2352,10 +2499,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L25" s="35" t="n"/>
+      <c r="L25" s="36" t="n"/>
+      <c r="M25" s="36" t="n"/>
+      <c r="N25" s="36" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="34" t="inlineStr">
+      <c r="A26" s="35" t="inlineStr">
         <is>
           <t>Short-read</t>
         </is>
@@ -2365,13 +2514,13 @@
           <t>Single-cell WGS (BioSkryb ResolveDNA)</t>
         </is>
       </c>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="35" t="n"/>
-      <c r="H26" s="35" t="n"/>
-      <c r="I26" s="35" t="n"/>
+      <c r="C26" s="36" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="36" t="n"/>
+      <c r="G26" s="36" t="n"/>
+      <c r="H26" s="36" t="n"/>
+      <c r="I26" s="36" t="n"/>
       <c r="J26" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2382,10 +2531,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L26" s="35" t="n"/>
+      <c r="L26" s="36" t="n"/>
+      <c r="M26" s="36" t="n"/>
+      <c r="N26" s="36" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="39" t="inlineStr">
+      <c r="A27" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2395,13 +2546,13 @@
           <t>Illumina bulk RNA-seq (mRNA + total RNA, UNC ×3 replicate)</t>
         </is>
       </c>
-      <c r="C27" s="35" t="n"/>
+      <c r="C27" s="36" t="n"/>
       <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E27" s="35" t="n"/>
+      <c r="E27" s="36" t="n"/>
       <c r="F27" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2412,14 +2563,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H27" s="35" t="n"/>
-      <c r="I27" s="35" t="n"/>
-      <c r="J27" s="35" t="n"/>
-      <c r="K27" s="35" t="n"/>
-      <c r="L27" s="35" t="n"/>
+      <c r="H27" s="36" t="n"/>
+      <c r="I27" s="36" t="n"/>
+      <c r="J27" s="36" t="n"/>
+      <c r="K27" s="36" t="n"/>
+      <c r="L27" s="36" t="n"/>
+      <c r="M27" s="36" t="n"/>
+      <c r="N27" s="36" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="39" t="inlineStr">
+      <c r="A28" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2429,13 +2582,13 @@
           <t>Illumina mRNA + lncRNA (Google/Novogene)</t>
         </is>
       </c>
-      <c r="C28" s="35" t="n"/>
+      <c r="C28" s="36" t="n"/>
       <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E28" s="35" t="n"/>
+      <c r="E28" s="36" t="n"/>
       <c r="F28" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2446,14 +2599,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H28" s="35" t="n"/>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="35" t="n"/>
-      <c r="K28" s="35" t="n"/>
-      <c r="L28" s="35" t="n"/>
+      <c r="H28" s="36" t="n"/>
+      <c r="I28" s="36" t="n"/>
+      <c r="J28" s="36" t="n"/>
+      <c r="K28" s="36" t="n"/>
+      <c r="L28" s="36" t="n"/>
+      <c r="M28" s="36" t="n"/>
+      <c r="N28" s="36" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="39" t="inlineStr">
+      <c r="A29" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2463,13 +2618,13 @@
           <t>PacBio Iso-Seq (Sequel II subreads, Google)</t>
         </is>
       </c>
-      <c r="C29" s="35" t="n"/>
+      <c r="C29" s="36" t="n"/>
       <c r="D29" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E29" s="35" t="n"/>
+      <c r="E29" s="36" t="n"/>
       <c r="F29" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2480,14 +2635,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H29" s="35" t="n"/>
-      <c r="I29" s="35" t="n"/>
-      <c r="J29" s="35" t="n"/>
-      <c r="K29" s="35" t="n"/>
-      <c r="L29" s="35" t="n"/>
+      <c r="H29" s="36" t="n"/>
+      <c r="I29" s="36" t="n"/>
+      <c r="J29" s="36" t="n"/>
+      <c r="K29" s="36" t="n"/>
+      <c r="L29" s="36" t="n"/>
+      <c r="M29" s="36" t="n"/>
+      <c r="N29" s="36" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2497,13 +2654,13 @@
           <t>PacBio MAS-Seq / Kinnex (full-length isoform)</t>
         </is>
       </c>
-      <c r="C30" s="35" t="n"/>
+      <c r="C30" s="36" t="n"/>
       <c r="D30" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E30" s="35" t="n"/>
+      <c r="E30" s="36" t="n"/>
       <c r="F30" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2514,14 +2671,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H30" s="35" t="n"/>
-      <c r="I30" s="35" t="n"/>
-      <c r="J30" s="35" t="n"/>
-      <c r="K30" s="35" t="n"/>
-      <c r="L30" s="35" t="n"/>
+      <c r="H30" s="36" t="n"/>
+      <c r="I30" s="36" t="n"/>
+      <c r="J30" s="36" t="n"/>
+      <c r="K30" s="36" t="n"/>
+      <c r="L30" s="36" t="n"/>
+      <c r="M30" s="36" t="n"/>
+      <c r="N30" s="36" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="39" t="inlineStr">
+      <c r="A31" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2531,13 +2690,13 @@
           <t>PacBio HiFi RNA (Baylor)</t>
         </is>
       </c>
-      <c r="C31" s="35" t="n"/>
+      <c r="C31" s="36" t="n"/>
       <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E31" s="35" t="n"/>
+      <c r="E31" s="36" t="n"/>
       <c r="F31" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2548,14 +2707,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H31" s="35" t="n"/>
-      <c r="I31" s="35" t="n"/>
-      <c r="J31" s="35" t="n"/>
-      <c r="K31" s="35" t="n"/>
-      <c r="L31" s="35" t="n"/>
+      <c r="H31" s="36" t="n"/>
+      <c r="I31" s="36" t="n"/>
+      <c r="J31" s="36" t="n"/>
+      <c r="K31" s="36" t="n"/>
+      <c r="L31" s="36" t="n"/>
+      <c r="M31" s="36" t="n"/>
+      <c r="N31" s="36" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="39" t="inlineStr">
+      <c r="A32" s="40" t="inlineStr">
         <is>
           <t>RNA-seq</t>
         </is>
@@ -2565,13 +2726,13 @@
           <t>ONT direct RNA (Mason)</t>
         </is>
       </c>
-      <c r="C32" s="35" t="n"/>
+      <c r="C32" s="36" t="n"/>
       <c r="D32" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E32" s="35" t="n"/>
+      <c r="E32" s="36" t="n"/>
       <c r="F32" s="20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2582,29 +2743,33 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H32" s="35" t="n"/>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="35" t="n"/>
-      <c r="K32" s="35" t="n"/>
-      <c r="L32" s="35" t="n"/>
+      <c r="H32" s="36" t="n"/>
+      <c r="I32" s="36" t="n"/>
+      <c r="J32" s="36" t="n"/>
+      <c r="K32" s="36" t="n"/>
+      <c r="L32" s="36" t="n"/>
+      <c r="M32" s="36" t="n"/>
+      <c r="N32" s="36" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="40" t="n"/>
-      <c r="B33" s="40" t="n"/>
-      <c r="C33" s="40" t="n"/>
-      <c r="D33" s="40" t="n"/>
-      <c r="E33" s="40" t="n"/>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="40" t="n"/>
-      <c r="H33" s="40" t="n"/>
-      <c r="I33" s="40" t="n"/>
-      <c r="J33" s="40" t="n"/>
-      <c r="K33" s="40" t="n"/>
-      <c r="L33" s="40" t="n"/>
+      <c r="A33" s="41" t="n"/>
+      <c r="B33" s="41" t="n"/>
+      <c r="C33" s="41" t="n"/>
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="41" t="n"/>
+      <c r="G33" s="41" t="n"/>
+      <c r="H33" s="41" t="n"/>
+      <c r="I33" s="41" t="n"/>
+      <c r="J33" s="41" t="n"/>
+      <c r="K33" s="41" t="n"/>
+      <c r="L33" s="41" t="n"/>
+      <c r="M33" s="41" t="n"/>
+      <c r="N33" s="41" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="40" t="n"/>
-      <c r="B34" s="41" t="inlineStr">
+      <c r="A34" s="41" t="n"/>
+      <c r="B34" s="42" t="inlineStr">
         <is>
           <t>플랫폼 수 (Y+L)</t>
         </is>
@@ -2649,20 +2814,30 @@
         <f>COUNTA(L5:L32)</f>
         <v/>
       </c>
+      <c r="M34" s="8">
+        <f>COUNTA(M5:M32)</f>
+        <v/>
+      </c>
+      <c r="N34" s="8">
+        <f>COUNTA(N5:N32)</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="40" t="n"/>
-      <c r="B35" s="40" t="n"/>
-      <c r="C35" s="40" t="n"/>
-      <c r="D35" s="40" t="n"/>
-      <c r="E35" s="40" t="n"/>
-      <c r="F35" s="40" t="n"/>
-      <c r="G35" s="40" t="n"/>
-      <c r="H35" s="40" t="n"/>
-      <c r="I35" s="40" t="n"/>
-      <c r="J35" s="40" t="n"/>
-      <c r="K35" s="40" t="n"/>
-      <c r="L35" s="40" t="n"/>
+      <c r="A35" s="41" t="n"/>
+      <c r="B35" s="41" t="n"/>
+      <c r="C35" s="41" t="n"/>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="41" t="n"/>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="41" t="n"/>
+      <c r="J35" s="41" t="n"/>
+      <c r="K35" s="41" t="n"/>
+      <c r="L35" s="41" t="n"/>
+      <c r="M35" s="41" t="n"/>
+      <c r="N35" s="41" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -2671,88 +2846,96 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="29" t="inlineStr">
         <is>
           <t>· 범례: Y = 데이터 제공, L = 제한적/일부, 빈칸 = 알려진 데이터 없음.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
+    <row r="38" ht="44" customHeight="1">
       <c r="A38" s="29" t="inlineStr">
         <is>
-          <t>· 이 시트는 2026-08-13 기준 GIAB FTP 전체 파일목록(current.tree, 86,392개)과 S3 버킷 실시간 목록(87,527개)을 대조해 검증했다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="28" customHeight="1">
+          <t>· 검증 방법: 2026-08-13 기준 GIAB FTP 전체 파일목록(current.tree, 86,392 files / 104.8 TiB)과 AWS S3 버킷 실시간 목록(87,527 objects / 118.1 TiB)을 대조하고, 샘플별 디렉토리는 FTP를 직접 조회해 확인했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1">
       <c r="A39" s="29" t="inlineStr">
         <is>
-          <t>· 2026-08-13 보정: SOLiD(HG001), Strand-seq(HG003~HG007), Hi-C(HG003·HG004), Element AVITI(HG001·HG003~HG005)를 빈칸에서 Y로 수정. BGISEQ/MGISEQ와 stLFR 행을 신규 추가(7개 germline 전체 제공).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="28" customHeight="1">
+          <t>· 2026-08-13 보정(DNA): SOLiD(HG001), Strand-seq(HG003~HG007), Hi-C(HG003·HG004), Element AVITI(HG001·HG003~HG005)를 빈칸에서 Y로 수정. BGISEQ-500/MGISEQ와 stLFR 행을 신규 추가했다(germline 7개 전체 제공).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1">
       <c r="A40" s="29" t="inlineStr">
         <is>
-          <t>· RNA-seq는 HG002·HG004·HG005 3개 샘플만 존재하며 총 6.5 TiB(324 files)다. HG001·HG003·HG006·HG007과 HG008(종양-정상)에는 RNA 데이터가 없다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
+          <t>· 2026-08-13 신규(HG009): data_somatic/HG009/ 에 두 번째 체세포 벤치마크가 추가되었다(2026-07 공개, 563 files / 1.5 TiB). 세포주 계대(passage)·클론 설계로 HG009-N은 WT-p4·WT-p25·LVTert-p23, HG009-T는 bulk p16·p42와 클론 6종(1C3·1D5·3C4·3C9·3F2·4G9)이며 현재 PacBio HiFi Revio(SPRQ)만 제공된다. NIST somatic WDL 분석 결과도 함께 배포된다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1">
       <c r="A41" s="29" t="inlineStr">
         <is>
-          <t>· 주의: RNA-seq 중 Illumina(UNC·Google)·Iso-Seq·Baylor HiFi RNA는 FTP에만 있고 AWS S3 미러에는 없다(6.3 TiB 누락). 이 데이터는 wget/FTP로 받아야 한다. MAS-Seq와 ONT direct RNA만 S3에 있다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="28" customHeight="1">
+          <t>· 2026-08-13 신규(HG008 확장): HG008-T 다른 계대(p2·p13) Illumina·ONT 데이터(other_passages, 1.2 TiB), HG008-N-D Illumina WGS(2025-11, 562 GiB), HG008-N-P Dovetail LinkPrep(2025-06, 209 GiB), HG002B Phase Genomics Hi-C(2024-10, 385 GiB)가 추가되었다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1">
       <c r="A42" s="29" t="inlineStr">
         <is>
-          <t>· 주의: germline DNA에서도 Element AVITI 2024-09(HG001~HG005, 약 2.1 TiB)는 S3 미러 누락 상태이며 FTP에서만 받을 수 있다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
+          <t>· RNA-seq는 HG002·HG004·HG005 3개 샘플만 존재하며 총 6.5 TiB(324 files)다. HG001·HG003·HG006·HG007과 HG008·HG009에는 RNA 데이터가 없다. 샘플별 용량은 HG002 3.9 TiB, HG004 1.4 TiB, HG005 1.4 TiB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="44" customHeight="1">
       <c r="A43" s="29" t="inlineStr">
         <is>
-          <t>· GIAB 공식 배포에 single-cell RNA-seq과 small RNA-seq(miRNA)은 없다. Single-cell은 DNA 기반(Strand-seq, BioSkryb)뿐이다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
+          <t>· 주의(S3 미러 누락): RNA-seq 중 Illumina(UNC·Google)·Iso-Seq·Baylor HiFi RNA는 FTP에만 있고 S3에는 없다(6.3 TiB). MAS-Seq와 ONT direct RNA만 S3에 있다. germline DNA에서도 Element AVITI 2024-09(HG001~HG005, 약 2.1 TiB)가 S3 미러 누락이다. 해당 데이터는 FTP(wget)로 받아야 한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="44" customHeight="1">
       <c r="A44" s="29" t="inlineStr">
         <is>
+          <t>· GIAB 공식 배포에 single-cell RNA-seq과 small RNA-seq(miRNA)은 없다. Single-cell은 DNA 기반(Strand-seq, BioSkryb ResolveDNA)뿐이다. Illumina RNA는 QC 리포트만 S3에 있고 raw는 FTP에서만 받을 수 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="44" customHeight="1">
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>· Methylation: PacBio HiFi 5mC는 germline(HG001·HG003~HG007)의 PacBio_CCS_15kb_20kb_chemistry2/GIAB_5mC_CpG/ 에 haplotagged BAM으로, HG008은 ONT dorado 5mC+5hmC modBAM으로 제공된다. WGBS/EM-seq은 GIAB에 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
           <t>· HG002는 사실상 모든 신규 플랫폼이 우선 적용되는 대표 샘플이고, trio 부모(HG003/4, HG006/7)는 일부 신규 플랫폼이 미적용이다.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="29" t="inlineStr">
-        <is>
-          <t>· HG008(종양-정상)은 2024~2025년 최신 기기 중심의 체세포 벤치마크로, 구형 플랫폼(SOLiD/CG/Ion 등)은 제공되지 않는다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="29" t="inlineStr">
-        <is>
-          <t>· 표준 GIAB 벤치마크 샘플은 HG001~HG008이며(HG008은 T·N-D·N-P의 3개 하위 시료), HG009 이상 신규 샘플은 확정·공표되지 않았다.</t>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>· HG008·HG009는 2024~2026년 최신 기기 중심의 체세포 벤치마크로, 구형 플랫폼(SOLiD/CG/Ion 등)은 제공되지 않는다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A38:L38"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A45:L45"/>
-    <mergeCell ref="A37:L37"/>
-    <mergeCell ref="A46:L46"/>
-    <mergeCell ref="A44:L44"/>
-    <mergeCell ref="A40:L40"/>
-    <mergeCell ref="A39:L39"/>
+  <mergeCells count="11">
+    <mergeCell ref="A40:N40"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="A38:N38"/>
+    <mergeCell ref="A46:N46"/>
+    <mergeCell ref="A43:N43"/>
+    <mergeCell ref="A41:N41"/>
+    <mergeCell ref="A47:N47"/>
+    <mergeCell ref="A42:N42"/>
+    <mergeCell ref="A37:N37"/>
+    <mergeCell ref="A44:N44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2764,7 +2947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3004,50 +3187,62 @@
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>추가 경로 (2026-08-13)</t>
+          <t>추가 경로 (2026-08-13 최신화)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="42" t="inlineStr">
-        <is>
-          <t>RNA-seq 데이터 FTP (HG002/HG004/HG005)</t>
-        </is>
-      </c>
-      <c r="B26" s="43" t="inlineStr">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>HG009 체세포 벤치마크 (신규, 2026-07)</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/data_somatic/HG009/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>RNA-seq 데이터 (HG002·HG004·HG005)</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="inlineStr">
         <is>
           <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/data_RNAseq/</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>AWS S3 미러 (일부 데이터 누락 — 아래 주의)</t>
-        </is>
-      </c>
-      <c r="B27" s="43" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="43" t="inlineStr">
+        <is>
+          <t>FTP 전체 파일목록 (크기·MD5 포함)</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/current.tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="43" t="inlineStr">
+        <is>
+          <t>AWS S3 미러 (일부 누락 — 아래 주의)</t>
+        </is>
+      </c>
+      <c r="B29" s="44" t="inlineStr">
         <is>
           <t>https://giab.s3.amazonaws.com/</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="42" t="inlineStr">
-        <is>
-          <t>FTP 전체 파일목록 (크기·MD5 포함)</t>
-        </is>
-      </c>
-      <c r="B28" s="43" t="inlineStr">
-        <is>
-          <t>https://ftp-trace.ncbi.nlm.nih.gov/ReferenceSamples/giab/current.tree</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="44" t="inlineStr">
-        <is>
-          <t>· S3 미러는 FTP보다 불완전하다. RNA-seq Illumina/Iso-Seq(6.3 TiB)과 Element AVITI 2024-09(2.1 TiB)은 S3에 없으므로 FTP(wget)로 받아야 한다.</t>
+    <row r="31">
+      <c r="A31" s="45" t="inlineStr">
+        <is>
+          <t>· S3 미러는 FTP보다 불완전하다. RNA-seq Illumina/Iso-Seq(6.3 TiB)과 Element AVITI 2024-09(2.1 TiB)은 S3에 없어 FTP(wget)로 받아야 한다.</t>
         </is>
       </c>
     </row>

</xml_diff>